<commit_message>
left side of tips & benefits title done
</commit_message>
<xml_diff>
--- a/assets/ExcelQuote.xlsx
+++ b/assets/ExcelQuote.xlsx
@@ -41,7 +41,27 @@
     <t xml:space="preserve">Dependant monthly cost</t>
   </si>
   <si>
-    <t xml:space="preserve">Total monthly cost (incl. employer subsidy)</t>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Total monthly cost</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (including employer subsidy)</t>
+    </r>
   </si>
   <si>
     <r>
@@ -57,7 +77,6 @@
     </r>
     <r>
       <rPr>
-        <b val="true"/>
         <i val="true"/>
         <sz val="14"/>
         <color rgb="FF000000"/>
@@ -65,62 +84,62 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(after employer subsidy)</t>
+      <t xml:space="preserve">(after subsidy)</t>
     </r>
   </si>
   <si>
     <t xml:space="preserve">YouPay</t>
   </si>
   <si>
-    <t xml:space="preserve">BasicsTitle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DeductibleLabel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DeductibleValue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BasicsLabel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BasicsValue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hospital StayTitle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hospital StayLabel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hospital StayValue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OutpatientTitle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OutpatientLabel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OutpatientValue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExtrasTitle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExtrasLabel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExtrasValue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DentalTitle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DentalLabel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DentalValue</t>
+    <t xml:space="preserve">Sec0Title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spec1Label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spec1Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec0Label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec0Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec1Title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec1Label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec1Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec2Title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec2Label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec2Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec3Title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec3Label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec3Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec4Title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec4Label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sec4Value</t>
   </si>
   <si>
     <t xml:space="preserve">TipTitle</t>
@@ -199,6 +218,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -220,7 +247,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <i val="true"/>
       <sz val="14"/>
       <color rgb="FF000000"/>
@@ -255,14 +281,6 @@
       <i val="true"/>
       <sz val="14"/>
       <color theme="3" tint="0.3999"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -456,7 +474,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -509,10 +527,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -521,23 +535,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -546,10 +556,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -561,7 +575,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -573,7 +587,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -585,7 +599,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="7" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -597,7 +611,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -700,9 +714,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>63360</xdr:colOff>
+      <xdr:colOff>63000</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>73440</xdr:rowOff>
+      <xdr:rowOff>73080</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -712,7 +726,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="7460640" y="3548520"/>
-          <a:ext cx="183960" cy="263880"/>
+          <a:ext cx="183600" cy="263520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -740,9 +754,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>2276280</xdr:colOff>
+      <xdr:colOff>2275920</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>1142640</xdr:rowOff>
+      <xdr:rowOff>1141200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -756,7 +770,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="3877200" cy="1142640"/>
+          <a:ext cx="3876840" cy="1141200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1036,134 +1050,134 @@
     </row>
     <row r="10" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="11" s="2" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="13"/>
-      <c r="D11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="J11" s="14"/>
-      <c r="L11" s="14"/>
+      <c r="B11" s="5"/>
+      <c r="D11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="J11" s="13"/>
+      <c r="L11" s="13"/>
     </row>
     <row r="12" s="2" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="13"/>
-      <c r="D12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="J12" s="14"/>
-      <c r="L12" s="14"/>
+      <c r="B12" s="5"/>
+      <c r="D12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="L12" s="13"/>
     </row>
     <row r="13" s="2" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B13" s="13"/>
-      <c r="D13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="J13" s="14"/>
-      <c r="L13" s="14"/>
+      <c r="B13" s="5"/>
+      <c r="D13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="J13" s="13"/>
+      <c r="L13" s="13"/>
     </row>
     <row r="14" s="2" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="13"/>
-      <c r="D14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="J14" s="14"/>
-      <c r="L14" s="14"/>
+      <c r="B14" s="5"/>
+      <c r="D14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="J14" s="13"/>
+      <c r="L14" s="13"/>
     </row>
     <row r="15" s="2" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B15" s="13"/>
-      <c r="D15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="J15" s="14"/>
-      <c r="L15" s="14"/>
+      <c r="B15" s="5"/>
+      <c r="D15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="J15" s="13"/>
+      <c r="L15" s="13"/>
     </row>
     <row r="16" s="2" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="13"/>
-      <c r="D16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="L16" s="14"/>
+      <c r="B16" s="5"/>
+      <c r="D16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="H16" s="13"/>
+      <c r="J16" s="13"/>
+      <c r="L16" s="13"/>
     </row>
     <row r="17" s="2" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="13"/>
-      <c r="D17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="L17" s="14"/>
+      <c r="B17" s="5"/>
+      <c r="D17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="J17" s="13"/>
+      <c r="L17" s="13"/>
     </row>
     <row r="18" s="2" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="13"/>
-      <c r="D18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="L18" s="14"/>
+      <c r="B18" s="5"/>
+      <c r="D18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="J18" s="13"/>
+      <c r="L18" s="13"/>
     </row>
     <row r="19" s="2" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="D19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="J19" s="14"/>
-      <c r="L19" s="14"/>
+      <c r="B19" s="5"/>
+      <c r="D19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="L19" s="13"/>
     </row>
     <row r="20" s="2" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B20" s="13"/>
-      <c r="D20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="J20" s="14"/>
-      <c r="L20" s="14"/>
-    </row>
-    <row r="21" s="2" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15" t="s">
+      <c r="B20" s="5"/>
+      <c r="D20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="L20" s="13"/>
+    </row>
+    <row r="21" s="2" customFormat="true" ht="19.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="H21" s="16"/>
-      <c r="J21" s="16"/>
-      <c r="L21" s="16"/>
-    </row>
-    <row r="22" s="2" customFormat="true" ht="23.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17" t="s">
+      <c r="D21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="J21" s="15"/>
+      <c r="L21" s="15"/>
+    </row>
+    <row r="22" s="2" customFormat="true" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="J22" s="18"/>
-      <c r="L22" s="18"/>
+      <c r="D22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="J22" s="17"/>
+      <c r="L22" s="17"/>
     </row>
     <row r="23" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="24" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1539,29 +1553,29 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="23.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="20" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="2"/>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="21" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="23"/>
-      <c r="C5" s="24" t="s">
+      <c r="B5" s="22"/>
+      <c r="C5" s="23" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="24" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1572,14 +1586,14 @@
       <c r="E6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="27" t="s">
+      <c r="C7" s="26" t="s">
         <v>15</v>
       </c>
       <c r="D7" s="2"/>
-      <c r="E7" s="28" t="s">
+      <c r="E7" s="27" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1590,14 +1604,14 @@
       <c r="E8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="26" t="s">
         <v>18</v>
       </c>
       <c r="D9" s="2"/>
-      <c r="E9" s="28" t="s">
+      <c r="E9" s="27" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1608,14 +1622,14 @@
       <c r="E10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="29" t="s">
+      <c r="B11" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="30" t="s">
+      <c r="C11" s="29" t="s">
         <v>21</v>
       </c>
       <c r="D11" s="2"/>
-      <c r="E11" s="31" t="s">
+      <c r="E11" s="30" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1626,37 +1640,37 @@
       <c r="E12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="33" t="s">
+      <c r="C13" s="32" t="s">
         <v>24</v>
       </c>
       <c r="D13" s="2"/>
-      <c r="E13" s="34" t="s">
+      <c r="E13" s="33" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="35" t="s">
+      <c r="B15" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="36" t="s">
+      <c r="E15" s="35" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="37" t="s">
+      <c r="B17" s="36" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="38" t="s">
+      <c r="B19" s="37" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="39" t="s">
+      <c r="B21" s="38" t="s">
         <v>30</v>
       </c>
     </row>

</xml_diff>